<commit_message>
chore: update notebooks and artifacts
</commit_message>
<xml_diff>
--- a/unit2-cleaning/examples/sample_data.xlsx
+++ b/unit2-cleaning/examples/sample_data.xlsx
@@ -334,16 +334,16 @@
     <t>Person_100</t>
   </si>
   <si>
+    <t>HR</t>
+  </si>
+  <si>
     <t>Sales</t>
   </si>
   <si>
+    <t>Finance</t>
+  </si>
+  <si>
     <t>IT</t>
-  </si>
-  <si>
-    <t>Finance</t>
-  </si>
-  <si>
-    <t>HR</t>
   </si>
 </sst>
 </file>
@@ -736,10 +736,10 @@
         <v>6</v>
       </c>
       <c r="C2">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="D2">
-        <v>48747.18225563578</v>
+        <v>70031.93318711054</v>
       </c>
       <c r="E2" t="s">
         <v>106</v>
@@ -756,13 +756,13 @@
         <v>7</v>
       </c>
       <c r="C3">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D3">
-        <v>30115.39204226672</v>
+        <v>44339.48615043852</v>
       </c>
       <c r="E3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F3" s="2">
         <v>43832</v>
@@ -776,13 +776,13 @@
         <v>8</v>
       </c>
       <c r="C4">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="D4">
-        <v>41748.34994549691</v>
+        <v>36412.24063263457</v>
       </c>
       <c r="E4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F4" s="2">
         <v>43833</v>
@@ -796,13 +796,13 @@
         <v>9</v>
       </c>
       <c r="C5">
-        <v>76</v>
+        <v>25</v>
       </c>
       <c r="D5">
-        <v>28919.53431584542</v>
+        <v>40633.92213535689</v>
       </c>
       <c r="E5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F5" s="2">
         <v>43834</v>
@@ -816,13 +816,13 @@
         <v>10</v>
       </c>
       <c r="C6">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="D6">
-        <v>47328.46828840613</v>
+        <v>55245.72117810347</v>
       </c>
       <c r="E6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F6" s="2">
         <v>43835</v>
@@ -836,13 +836,13 @@
         <v>11</v>
       </c>
       <c r="C7">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="D7">
-        <v>27633.67032192531</v>
+        <v>56995.98719900852</v>
       </c>
       <c r="E7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F7" s="2">
         <v>43836</v>
@@ -856,10 +856,10 @@
         <v>12</v>
       </c>
       <c r="C8">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="D8">
-        <v>38923.80875683604</v>
+        <v>41313.65040119455</v>
       </c>
       <c r="E8" t="s">
         <v>108</v>
@@ -876,13 +876,13 @@
         <v>13</v>
       </c>
       <c r="C9">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D9">
-        <v>66166.54689679258</v>
+        <v>39704.00812983613</v>
       </c>
       <c r="E9" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F9" s="2">
         <v>43838</v>
@@ -896,13 +896,13 @@
         <v>14</v>
       </c>
       <c r="C10">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="D10">
-        <v>42229.91875356604</v>
+        <v>71880.98548923334</v>
       </c>
       <c r="E10" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F10" s="2">
         <v>43839</v>
@@ -916,13 +916,13 @@
         <v>15</v>
       </c>
       <c r="C11">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="D11">
-        <v>53676.41526129905</v>
+        <v>45147.84131530975</v>
       </c>
       <c r="E11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F11" s="2">
         <v>43840</v>
@@ -936,13 +936,13 @@
         <v>16</v>
       </c>
       <c r="C12">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D12">
-        <v>54608.44877630944</v>
+        <v>42540.89982205989</v>
       </c>
       <c r="E12" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F12" s="2">
         <v>43841</v>
@@ -956,10 +956,10 @@
         <v>17</v>
       </c>
       <c r="C13">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="D13">
-        <v>44604.76962374042</v>
+        <v>27634.41540442471</v>
       </c>
       <c r="E13" t="s">
         <v>107</v>
@@ -976,10 +976,10 @@
         <v>18</v>
       </c>
       <c r="C14">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="D14">
-        <v>62124.99708616879</v>
+        <v>104321.2053833028</v>
       </c>
       <c r="E14" t="s">
         <v>108</v>
@@ -996,10 +996,10 @@
         <v>19</v>
       </c>
       <c r="C15">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D15">
-        <v>62627.20076670023</v>
+        <v>26379.64128967778</v>
       </c>
       <c r="E15" t="s">
         <v>108</v>
@@ -1016,10 +1016,10 @@
         <v>20</v>
       </c>
       <c r="C16">
-        <v>24</v>
+        <v>68</v>
       </c>
       <c r="D16">
-        <v>59138.32754534869</v>
+        <v>47582.83895733198</v>
       </c>
       <c r="E16" t="s">
         <v>108</v>
@@ -1036,10 +1036,10 @@
         <v>21</v>
       </c>
       <c r="C17">
-        <v>62</v>
+        <v>18</v>
       </c>
       <c r="D17">
-        <v>33641.82103386788</v>
+        <v>68384.62396623399</v>
       </c>
       <c r="E17" t="s">
         <v>109</v>
@@ -1056,10 +1056,10 @@
         <v>22</v>
       </c>
       <c r="C18">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="D18">
-        <v>49043.63139532429</v>
+        <v>61084.36803841175</v>
       </c>
       <c r="E18" t="s">
         <v>106</v>
@@ -1076,13 +1076,13 @@
         <v>23</v>
       </c>
       <c r="C19">
-        <v>21</v>
+        <v>67</v>
       </c>
       <c r="D19">
-        <v>56847.59821639571</v>
+        <v>31146.56983622814</v>
       </c>
       <c r="E19" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F19" s="2">
         <v>43848</v>
@@ -1096,10 +1096,10 @@
         <v>24</v>
       </c>
       <c r="C20">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D20">
-        <v>42274.05384377464</v>
+        <v>45445.61408060648</v>
       </c>
       <c r="E20" t="s">
         <v>107</v>
@@ -1116,13 +1116,13 @@
         <v>25</v>
       </c>
       <c r="C21">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="D21">
-        <v>68393.99577512604</v>
+        <v>39905.9474576351</v>
       </c>
       <c r="E21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F21" s="2">
         <v>43850</v>
@@ -1136,13 +1136,13 @@
         <v>26</v>
       </c>
       <c r="C22">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="D22">
-        <v>46966.98717729333</v>
+        <v>46157.03545827596</v>
       </c>
       <c r="E22" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F22" s="2">
         <v>43851</v>
@@ -1156,10 +1156,10 @@
         <v>27</v>
       </c>
       <c r="C23">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="D23">
-        <v>45037.35445987143</v>
+        <v>47094.71839907426</v>
       </c>
       <c r="E23" t="s">
         <v>108</v>
@@ -1176,13 +1176,13 @@
         <v>28</v>
       </c>
       <c r="C24">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="D24">
-        <v>25125.24721837497</v>
+        <v>38082.18236910208</v>
       </c>
       <c r="E24" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F24" s="2">
         <v>43853</v>
@@ -1196,13 +1196,13 @@
         <v>29</v>
       </c>
       <c r="C25">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="D25">
-        <v>29474.0067394532</v>
+        <v>81645.81570803224</v>
       </c>
       <c r="E25" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F25" s="2">
         <v>43854</v>
@@ -1216,13 +1216,13 @@
         <v>30</v>
       </c>
       <c r="C26">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D26">
-        <v>58712.33365640082</v>
+        <v>40564.22916246224</v>
       </c>
       <c r="E26" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F26" s="2">
         <v>43855</v>
@@ -1236,13 +1236,13 @@
         <v>31</v>
       </c>
       <c r="C27">
-        <v>48</v>
+        <v>19</v>
       </c>
       <c r="D27">
-        <v>70269.52866785933</v>
+        <v>53210.77687804967</v>
       </c>
       <c r="E27" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F27" s="2">
         <v>43856</v>
@@ -1256,13 +1256,13 @@
         <v>32</v>
       </c>
       <c r="C28">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D28">
-        <v>56227.08707745132</v>
+        <v>28628.02826795025</v>
       </c>
       <c r="E28" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F28" s="2">
         <v>43857</v>
@@ -1276,13 +1276,13 @@
         <v>33</v>
       </c>
       <c r="C29">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="D29">
-        <v>63885.03663094122</v>
+        <v>20262.05446624028</v>
       </c>
       <c r="E29" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F29" s="2">
         <v>43858</v>
@@ -1296,13 +1296,13 @@
         <v>34</v>
       </c>
       <c r="C30">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="D30">
-        <v>52077.74816613758</v>
+        <v>44988.47536353441</v>
       </c>
       <c r="E30" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F30" s="2">
         <v>43859</v>
@@ -1316,10 +1316,10 @@
         <v>35</v>
       </c>
       <c r="C31">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="D31">
-        <v>42505.01488833394</v>
+        <v>50945.65627707195</v>
       </c>
       <c r="E31" t="s">
         <v>109</v>
@@ -1336,13 +1336,13 @@
         <v>36</v>
       </c>
       <c r="C32">
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="D32">
-        <v>58338.250549846</v>
+        <v>46104.89441809453</v>
       </c>
       <c r="E32" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F32" s="2">
         <v>43861</v>
@@ -1356,13 +1356,13 @@
         <v>37</v>
       </c>
       <c r="C33">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D33">
-        <v>58961.62394646474</v>
+        <v>43160.75284155552</v>
       </c>
       <c r="E33" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F33" s="2">
         <v>43862</v>
@@ -1376,13 +1376,13 @@
         <v>38</v>
       </c>
       <c r="C34">
-        <v>78</v>
+        <v>33</v>
       </c>
       <c r="D34">
-        <v>50474.76445185542</v>
+        <v>96621.68775170541</v>
       </c>
       <c r="E34" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F34" s="2">
         <v>43863</v>
@@ -1396,13 +1396,13 @@
         <v>39</v>
       </c>
       <c r="C35">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="D35">
-        <v>45200.74095117793</v>
+        <v>44929.68511239845</v>
       </c>
       <c r="E35" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F35" s="2">
         <v>43864</v>
@@ -1416,13 +1416,13 @@
         <v>40</v>
       </c>
       <c r="C36">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="D36">
-        <v>76871.29837205488</v>
+        <v>69246.2684317994</v>
       </c>
       <c r="E36" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F36" s="2">
         <v>43865</v>
@@ -1436,13 +1436,13 @@
         <v>41</v>
       </c>
       <c r="C37">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D37">
-        <v>53810.28041161156</v>
+        <v>73031.90511954107</v>
       </c>
       <c r="E37" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F37" s="2">
         <v>43866</v>
@@ -1456,13 +1456,13 @@
         <v>42</v>
       </c>
       <c r="C38">
-        <v>27</v>
+        <v>74</v>
       </c>
       <c r="D38">
-        <v>43970.71778374718</v>
+        <v>49524.28380312018</v>
       </c>
       <c r="E38" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F38" s="2">
         <v>43867</v>
@@ -1476,13 +1476,13 @@
         <v>43</v>
       </c>
       <c r="C39">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="D39">
-        <v>50066.52584702597</v>
+        <v>69177.23846854286</v>
       </c>
       <c r="E39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F39" s="2">
         <v>43868</v>
@@ -1496,13 +1496,13 @@
         <v>44</v>
       </c>
       <c r="C40">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D40">
-        <v>50628.88656703735</v>
+        <v>43053.5650965731</v>
       </c>
       <c r="E40" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F40" s="2">
         <v>43869</v>
@@ -1516,13 +1516,13 @@
         <v>45</v>
       </c>
       <c r="C41">
-        <v>67</v>
+        <v>19</v>
       </c>
       <c r="D41">
-        <v>35728.47694440125</v>
+        <v>37985.2583119807</v>
       </c>
       <c r="E41" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F41" s="2">
         <v>43870</v>
@@ -1536,13 +1536,13 @@
         <v>46</v>
       </c>
       <c r="C42">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="D42">
-        <v>46194.82902647479</v>
+        <v>43949.67862793499</v>
       </c>
       <c r="E42" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F42" s="2">
         <v>43871</v>
@@ -1556,13 +1556,13 @@
         <v>47</v>
       </c>
       <c r="C43">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D43">
-        <v>85882.90804363557</v>
+        <v>34451.61935501292</v>
       </c>
       <c r="E43" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F43" s="2">
         <v>43872</v>
@@ -1576,13 +1576,13 @@
         <v>48</v>
       </c>
       <c r="C44">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="D44">
-        <v>81673.83793967988</v>
+        <v>57266.40451495141</v>
       </c>
       <c r="E44" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F44" s="2">
         <v>43873</v>
@@ -1596,13 +1596,13 @@
         <v>49</v>
       </c>
       <c r="C45">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="D45">
-        <v>51089.47488489129</v>
+        <v>51297.11833200431</v>
       </c>
       <c r="E45" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F45" s="2">
         <v>43874</v>
@@ -1616,13 +1616,13 @@
         <v>50</v>
       </c>
       <c r="C46">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="D46">
-        <v>17160.39650100514</v>
+        <v>24688.54035215417</v>
       </c>
       <c r="E46" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F46" s="2">
         <v>43875</v>
@@ -1636,13 +1636,13 @@
         <v>51</v>
       </c>
       <c r="C47">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="D47">
-        <v>61563.04219691779</v>
+        <v>34722.55260820875</v>
       </c>
       <c r="E47" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F47" s="2">
         <v>43876</v>
@@ -1656,10 +1656,10 @@
         <v>52</v>
       </c>
       <c r="C48">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="D48">
-        <v>53360.38571940515</v>
+        <v>23289.31338311951</v>
       </c>
       <c r="E48" t="s">
         <v>106</v>
@@ -1676,10 +1676,10 @@
         <v>53</v>
       </c>
       <c r="C49">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="D49">
-        <v>51008.23630018337</v>
+        <v>64906.94457688379</v>
       </c>
       <c r="E49" t="s">
         <v>109</v>
@@ -1696,10 +1696,10 @@
         <v>54</v>
       </c>
       <c r="C50">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="D50">
-        <v>47948.04113218602</v>
+        <v>22458.33565283434</v>
       </c>
       <c r="E50" t="s">
         <v>106</v>
@@ -1716,13 +1716,13 @@
         <v>55</v>
       </c>
       <c r="C51">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="D51">
-        <v>67014.63247384084</v>
+        <v>60973.54001693003</v>
       </c>
       <c r="E51" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F51" s="2">
         <v>43880</v>
@@ -1736,13 +1736,13 @@
         <v>56</v>
       </c>
       <c r="C52">
-        <v>77</v>
+        <v>38</v>
       </c>
       <c r="D52">
-        <v>70709.92284020971</v>
+        <v>50381.71255760929</v>
       </c>
       <c r="E52" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F52" s="2">
         <v>43881</v>
@@ -1756,13 +1756,13 @@
         <v>57</v>
       </c>
       <c r="C53">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="D53">
-        <v>44823.78157863708</v>
+        <v>26192.56416357059</v>
       </c>
       <c r="E53" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F53" s="2">
         <v>43882</v>
@@ -1776,13 +1776,13 @@
         <v>58</v>
       </c>
       <c r="C54">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D54">
-        <v>44311.38369641478</v>
+        <v>27889.42337767935</v>
       </c>
       <c r="E54" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F54" s="2">
         <v>43883</v>
@@ -1796,13 +1796,13 @@
         <v>59</v>
       </c>
       <c r="C55">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="D55">
-        <v>56194.24908299612</v>
+        <v>25309.81445702696</v>
       </c>
       <c r="E55" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F55" s="2">
         <v>43884</v>
@@ -1816,13 +1816,13 @@
         <v>60</v>
       </c>
       <c r="C56">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D56">
-        <v>62691.97149345225</v>
+        <v>53219.04044541816</v>
       </c>
       <c r="E56" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F56" s="2">
         <v>43885</v>
@@ -1836,10 +1836,10 @@
         <v>61</v>
       </c>
       <c r="C57">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="D57">
-        <v>43975.33382417331</v>
+        <v>30024.49121833482</v>
       </c>
       <c r="E57" t="s">
         <v>107</v>
@@ -1856,10 +1856,10 @@
         <v>62</v>
       </c>
       <c r="C58">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="D58">
-        <v>45875.84727537336</v>
+        <v>60930.98582832234</v>
       </c>
       <c r="E58" t="s">
         <v>107</v>
@@ -1876,13 +1876,13 @@
         <v>63</v>
       </c>
       <c r="C59">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="D59">
-        <v>52935.84542437725</v>
+        <v>11698.29601518893</v>
       </c>
       <c r="E59" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F59" s="2">
         <v>43888</v>
@@ -1896,13 +1896,13 @@
         <v>64</v>
       </c>
       <c r="C60">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="D60">
-        <v>45230.50155226173</v>
+        <v>45876.28229020657</v>
       </c>
       <c r="E60" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F60" s="2">
         <v>43889</v>
@@ -1916,13 +1916,13 @@
         <v>65</v>
       </c>
       <c r="C61">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="D61">
-        <v>46375.19437984942</v>
+        <v>42568.54140811945</v>
       </c>
       <c r="E61" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F61" s="2">
         <v>43890</v>
@@ -1936,13 +1936,13 @@
         <v>66</v>
       </c>
       <c r="C62">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="D62">
-        <v>81805.78806199362</v>
+        <v>22772.14220536061</v>
       </c>
       <c r="E62" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F62" s="2">
         <v>43891</v>
@@ -1956,13 +1956,13 @@
         <v>67</v>
       </c>
       <c r="C63">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="D63">
-        <v>51958.882278378</v>
+        <v>55753.04944641775</v>
       </c>
       <c r="E63" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F63" s="2">
         <v>43892</v>
@@ -1976,10 +1976,10 @@
         <v>68</v>
       </c>
       <c r="C64">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="D64">
-        <v>60772.7495886137</v>
+        <v>54770.04606641386</v>
       </c>
       <c r="E64" t="s">
         <v>106</v>
@@ -1996,10 +1996,10 @@
         <v>69</v>
       </c>
       <c r="C65">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="D65">
-        <v>72523.1779111428</v>
+        <v>54266.57571515262</v>
       </c>
       <c r="E65" t="s">
         <v>107</v>
@@ -2016,13 +2016,13 @@
         <v>70</v>
       </c>
       <c r="C66">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="D66">
-        <v>54409.09634286517</v>
+        <v>50633.10757389641</v>
       </c>
       <c r="E66" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F66" s="2">
         <v>43895</v>
@@ -2036,13 +2036,13 @@
         <v>71</v>
       </c>
       <c r="C67">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="D67">
-        <v>71138.43177575147</v>
+        <v>44522.14280996377</v>
       </c>
       <c r="E67" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F67" s="2">
         <v>43896</v>
@@ -2056,10 +2056,10 @@
         <v>72</v>
       </c>
       <c r="C68">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D68">
-        <v>58002.39667828627</v>
+        <v>43506.15359829836</v>
       </c>
       <c r="E68" t="s">
         <v>106</v>
@@ -2076,10 +2076,10 @@
         <v>73</v>
       </c>
       <c r="C69">
-        <v>29</v>
+        <v>72</v>
       </c>
       <c r="D69">
-        <v>42229.13039219988</v>
+        <v>39231.36971731714</v>
       </c>
       <c r="E69" t="s">
         <v>106</v>
@@ -2096,13 +2096,13 @@
         <v>74</v>
       </c>
       <c r="C70">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="D70">
-        <v>33100.17028626416</v>
+        <v>28622.17443828121</v>
       </c>
       <c r="E70" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F70" s="2">
         <v>43899</v>
@@ -2116,13 +2116,13 @@
         <v>75</v>
       </c>
       <c r="C71">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="D71">
-        <v>35927.28971255108</v>
+        <v>46660.13403475525</v>
       </c>
       <c r="E71" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F71" s="2">
         <v>43900</v>
@@ -2136,10 +2136,10 @@
         <v>76</v>
       </c>
       <c r="C72">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="D72">
-        <v>79779.14480813245</v>
+        <v>55269.14279486284</v>
       </c>
       <c r="E72" t="s">
         <v>106</v>
@@ -2156,13 +2156,13 @@
         <v>77</v>
       </c>
       <c r="C73">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="D73">
-        <v>62753.8276106726</v>
+        <v>49369.31793091312</v>
       </c>
       <c r="E73" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F73" s="2">
         <v>43902</v>
@@ -2176,13 +2176,13 @@
         <v>78</v>
       </c>
       <c r="C74">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D74">
-        <v>44413.54666275848</v>
+        <v>52634.70491450026</v>
       </c>
       <c r="E74" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F74" s="2">
         <v>43903</v>
@@ -2196,13 +2196,13 @@
         <v>79</v>
       </c>
       <c r="C75">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="D75">
-        <v>60504.17068824657</v>
+        <v>58093.07268541645</v>
       </c>
       <c r="E75" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F75" s="2">
         <v>43904</v>
@@ -2216,13 +2216,13 @@
         <v>80</v>
       </c>
       <c r="C76">
-        <v>49</v>
+        <v>74</v>
       </c>
       <c r="D76">
-        <v>69815.43867979474</v>
+        <v>21104.83362102615</v>
       </c>
       <c r="E76" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F76" s="2">
         <v>43905</v>
@@ -2236,10 +2236,10 @@
         <v>81</v>
       </c>
       <c r="C77">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="D77">
-        <v>49570.44601291049</v>
+        <v>47002.04081502084</v>
       </c>
       <c r="E77" t="s">
         <v>109</v>
@@ -2256,13 +2256,13 @@
         <v>82</v>
       </c>
       <c r="C78">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D78">
-        <v>62552.59644420939</v>
+        <v>43522.73354116231</v>
       </c>
       <c r="E78" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F78" s="2">
         <v>43907</v>
@@ -2276,13 +2276,13 @@
         <v>83</v>
       </c>
       <c r="C79">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D79">
-        <v>60999.36650136659</v>
+        <v>52651.02191396571</v>
       </c>
       <c r="E79" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F79" s="2">
         <v>43908</v>
@@ -2296,13 +2296,13 @@
         <v>84</v>
       </c>
       <c r="C80">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="D80">
-        <v>42116.29517962358</v>
+        <v>69856.54032681164</v>
       </c>
       <c r="E80" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F80" s="2">
         <v>43909</v>
@@ -2316,13 +2316,13 @@
         <v>85</v>
       </c>
       <c r="C81">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D81">
-        <v>47480.33511445128</v>
+        <v>49734.0561144293</v>
       </c>
       <c r="E81" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F81" s="2">
         <v>43910</v>
@@ -2336,10 +2336,10 @@
         <v>86</v>
       </c>
       <c r="C82">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="D82">
-        <v>67210.72666778362</v>
+        <v>59912.5350895669</v>
       </c>
       <c r="E82" t="s">
         <v>108</v>
@@ -2356,13 +2356,13 @@
         <v>87</v>
       </c>
       <c r="C83">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="D83">
-        <v>42132.27539997448</v>
+        <v>40598.14206985763</v>
       </c>
       <c r="E83" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F83" s="2">
         <v>43912</v>
@@ -2376,13 +2376,13 @@
         <v>88</v>
       </c>
       <c r="C84">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="D84">
-        <v>45738.73883513115</v>
+        <v>69409.57579550729</v>
       </c>
       <c r="E84" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F84" s="2">
         <v>43913</v>
@@ -2396,13 +2396,13 @@
         <v>89</v>
       </c>
       <c r="C85">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="D85">
-        <v>66469.08386290674</v>
+        <v>39472.96299795101</v>
       </c>
       <c r="E85" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F85" s="2">
         <v>43914</v>
@@ -2416,10 +2416,10 @@
         <v>90</v>
       </c>
       <c r="C86">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="D86">
-        <v>40558.44006106135</v>
+        <v>63844.11464024072</v>
       </c>
       <c r="E86" t="s">
         <v>106</v>
@@ -2436,13 +2436,13 @@
         <v>91</v>
       </c>
       <c r="C87">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="D87">
-        <v>34384.61200073149</v>
+        <v>39825.11621064194</v>
       </c>
       <c r="E87" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F87" s="2">
         <v>43916</v>
@@ -2456,13 +2456,13 @@
         <v>92</v>
       </c>
       <c r="C88">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="D88">
-        <v>63132.1742196581</v>
+        <v>44782.38138141281</v>
       </c>
       <c r="E88" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F88" s="2">
         <v>43917</v>
@@ -2476,13 +2476,13 @@
         <v>93</v>
       </c>
       <c r="C89">
-        <v>32</v>
+        <v>76</v>
       </c>
       <c r="D89">
-        <v>44166.57388944553</v>
+        <v>44912.84936836828</v>
       </c>
       <c r="E89" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F89" s="2">
         <v>43918</v>
@@ -2496,13 +2496,13 @@
         <v>94</v>
       </c>
       <c r="C90">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="D90">
-        <v>49508.16176961461</v>
+        <v>50982.04265420557</v>
       </c>
       <c r="E90" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F90" s="2">
         <v>43919</v>
@@ -2516,13 +2516,13 @@
         <v>95</v>
       </c>
       <c r="C91">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="D91">
-        <v>70411.33857364788</v>
+        <v>37958.79512691291</v>
       </c>
       <c r="E91" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F91" s="2">
         <v>43920</v>
@@ -2536,13 +2536,13 @@
         <v>96</v>
       </c>
       <c r="C92">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D92">
-        <v>45340.90359442343</v>
+        <v>41582.54009652876</v>
       </c>
       <c r="E92" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F92" s="2">
         <v>43921</v>
@@ -2556,13 +2556,13 @@
         <v>97</v>
       </c>
       <c r="C93">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="D93">
-        <v>61177.84262268715</v>
+        <v>28827.43912696467</v>
       </c>
       <c r="E93" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F93" s="2">
         <v>43922</v>
@@ -2576,10 +2576,10 @@
         <v>98</v>
       </c>
       <c r="C94">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="D94">
-        <v>34253.9722916211</v>
+        <v>35850.30949534002</v>
       </c>
       <c r="E94" t="s">
         <v>107</v>
@@ -2596,13 +2596,13 @@
         <v>99</v>
       </c>
       <c r="C95">
-        <v>37</v>
+        <v>79</v>
       </c>
       <c r="D95">
-        <v>76485.02388135628</v>
+        <v>54679.41733581582</v>
       </c>
       <c r="E95" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F95" s="2">
         <v>43924</v>
@@ -2616,13 +2616,13 @@
         <v>100</v>
       </c>
       <c r="C96">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="D96">
-        <v>57601.53122227205</v>
+        <v>43792.01916811273</v>
       </c>
       <c r="E96" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F96" s="2">
         <v>43925</v>
@@ -2636,10 +2636,10 @@
         <v>101</v>
       </c>
       <c r="C97">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="D97">
-        <v>45945.4847975202</v>
+        <v>33762.08577916746</v>
       </c>
       <c r="E97" t="s">
         <v>108</v>
@@ -2656,13 +2656,13 @@
         <v>102</v>
       </c>
       <c r="C98">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="D98">
-        <v>70612.09564442124</v>
+        <v>72125.42147294918</v>
       </c>
       <c r="E98" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F98" s="2">
         <v>43927</v>
@@ -2676,13 +2676,13 @@
         <v>103</v>
       </c>
       <c r="C99">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="D99">
-        <v>59292.41802552177</v>
+        <v>77382.32596537781</v>
       </c>
       <c r="E99" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F99" s="2">
         <v>43928</v>
@@ -2696,13 +2696,13 @@
         <v>104</v>
       </c>
       <c r="C100">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="D100">
-        <v>51979.50292369697</v>
+        <v>81306.47256340373</v>
       </c>
       <c r="E100" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F100" s="2">
         <v>43929</v>
@@ -2716,13 +2716,13 @@
         <v>105</v>
       </c>
       <c r="C101">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D101">
-        <v>42914.25124921309</v>
+        <v>22974.49737146377</v>
       </c>
       <c r="E101" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F101" s="2">
         <v>43930</v>

</xml_diff>